<commit_message>
started random loot method for chest and made a seoarate file for testing
</commit_message>
<xml_diff>
--- a/assets/lists/item_list.xlsx
+++ b/assets/lists/item_list.xlsx
@@ -3,13 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ECF50D3-3202-4CB2-A5C5-770F0AF35687}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3EA23A3-CEC7-41AF-905E-43F1182A5171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ItemList" sheetId="1" r:id="rId1"/>
-    <sheet name="Notes" sheetId="2" r:id="rId2"/>
+    <sheet name="ChestDrops" sheetId="3" r:id="rId2"/>
+    <sheet name="Notes" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="80">
   <si>
     <t>halberd</t>
   </si>
@@ -255,6 +256,12 @@
   </si>
   <si>
     <t>sample</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Drop Rate</t>
   </si>
 </sst>
 </file>
@@ -344,7 +351,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -385,6 +392,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1895,6 +1903,391 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCE518B4-1F54-4508-A7E7-A2A853CAD793}">
+  <dimension ref="A1:C34"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1">
+        <v>128500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1">
+        <v>161400</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" s="1">
+        <v>166700</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5" s="1">
+        <v>151800</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6" s="1">
+        <v>162000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7">
+        <v>3</v>
+      </c>
+      <c r="C7" s="1">
+        <v>152300</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" s="1">
+        <v>144500</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9">
+        <v>3</v>
+      </c>
+      <c r="C9" s="1">
+        <v>145100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" s="1">
+        <v>125800</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11">
+        <v>3</v>
+      </c>
+      <c r="C11" s="1">
+        <v>136800</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12">
+        <v>3</v>
+      </c>
+      <c r="C12" s="1">
+        <v>153200</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" s="1">
+        <v>143600</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14" s="1">
+        <v>167100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+      <c r="C15" s="1">
+        <v>157200</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16" s="1">
+        <v>138000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" s="1">
+        <v>135400</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18">
+        <v>3</v>
+      </c>
+      <c r="C18" s="1">
+        <v>161700</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19">
+        <v>3</v>
+      </c>
+      <c r="C19" s="16">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20">
+        <v>3</v>
+      </c>
+      <c r="C20" s="16">
+        <v>200001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21">
+        <v>3</v>
+      </c>
+      <c r="C21" s="16">
+        <v>200002</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22">
+        <v>3</v>
+      </c>
+      <c r="C22" s="16">
+        <v>200003</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>16</v>
+      </c>
+      <c r="B23">
+        <v>3</v>
+      </c>
+      <c r="C23" s="16">
+        <v>200004</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24">
+        <v>3</v>
+      </c>
+      <c r="C24" s="16">
+        <v>200005</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>18</v>
+      </c>
+      <c r="B25">
+        <v>3</v>
+      </c>
+      <c r="C25" s="16">
+        <v>200006</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>19</v>
+      </c>
+      <c r="B26">
+        <v>3</v>
+      </c>
+      <c r="C26" s="16">
+        <v>200007</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B27">
+        <v>3</v>
+      </c>
+      <c r="C27" s="16">
+        <v>200008</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>21</v>
+      </c>
+      <c r="B28">
+        <v>3</v>
+      </c>
+      <c r="C28" s="16">
+        <v>200009</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>22</v>
+      </c>
+      <c r="B29">
+        <v>3</v>
+      </c>
+      <c r="C29" s="16">
+        <v>200010</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>23</v>
+      </c>
+      <c r="B30">
+        <v>3</v>
+      </c>
+      <c r="C30" s="16">
+        <v>200011</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>24</v>
+      </c>
+      <c r="B31">
+        <v>3</v>
+      </c>
+      <c r="C31" s="16">
+        <v>200012</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>25</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" s="16">
+        <v>200013</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>26</v>
+      </c>
+      <c r="B33">
+        <v>3</v>
+      </c>
+      <c r="C33" s="16">
+        <v>200014</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>27</v>
+      </c>
+      <c r="B34">
+        <v>3</v>
+      </c>
+      <c r="C34" s="16">
+        <v>200015</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C316504E-A4CF-4FFE-BF92-734B59BDD790}">
   <dimension ref="A2:F21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>